<commit_message>
Rebuild the PZ Nigeria files in Office 2013's default style
The deck is now built with python-pptx on PowerPoint 2013's widescreen
Office Theme (office2013.py converts python-pptx's template: Calibri
Light titles, Calibri text, the 2013 palette and placeholder positions)
using the standard layouts, with Table Grid tables and grey charts in
the content placeholders. The workbook uses the Office 2013 theme,
Calibri 11, grey header rows, black borders, gridlines and Excel 2013's
default chart style. Same content, transitions and animations.

sanitize_charts.py keeps chart axis ids in 1..2^31-1 (python-pptx
writes negative ids; ids above 2^31-1 lose their axes in some readers),
and validate_strict.py checks for it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WToQxHdrdWhM7bKqXvUa59
</commit_message>
<xml_diff>
--- a/pz-analysis/PZ_Nigeria_Analysis.xlsx
+++ b/pz-analysis/PZ_Nigeria_Analysis.xlsx
@@ -24,77 +24,48 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="5">
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="10"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <color rgb="00000000"/>
+      <sz val="14"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <i val="1"/>
-      <color rgb="00404040"/>
-      <sz val="10"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00404040"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00404040"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -103,30 +74,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-        <bgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DEEBF7"/>
-        <bgColor rgb="00DEEBF7"/>
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -136,39 +89,25 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="medium">
-        <color rgb="001F3864"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -177,109 +116,42 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -367,19 +239,19 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1200" b="1">
+              <a:defRPr sz="1400" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1200" b="1">
+              <a:rPr sz="1400" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:rPr>
               <a:t>Average PESTLE Score by Factor (out of 25)</a:t>
             </a:r>
@@ -421,21 +293,21 @@
             <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
             <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:pPr>
-                <a:defRPr sz="900" b="1">
+                <a:defRPr sz="900" b="0">
                   <a:solidFill>
-                    <a:srgbClr val="000000"/>
+                    <a:srgbClr val="404040"/>
                   </a:solidFill>
-                  <a:latin typeface="Arial"/>
+                  <a:latin typeface="+mn-lt"/>
                 </a:defRPr>
               </a:pPr>
               <a:r>
                 <a:t/>
               </a:r>
-              <a:endParaRPr sz="900" b="1">
+              <a:endParaRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="404040"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:endParaRPr>
             </a:p>
           </txPr>
@@ -446,7 +318,7 @@
           <showSerName val="0"/>
           <showPercent val="0"/>
         </dLbls>
-        <gapWidth val="60"/>
+        <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -462,7 +334,7 @@
         <spPr>
           <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
             <a:solidFill>
-              <a:srgbClr val="A6A6A6"/>
+              <a:srgbClr val="D9D9D9"/>
             </a:solidFill>
             <a:prstDash val="solid"/>
           </a:ln>
@@ -473,9 +345,9 @@
             <a:pPr>
               <a:defRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
@@ -483,9 +355,9 @@
             </a:r>
             <a:endParaRPr sz="900" b="0">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
-              <a:latin typeface="Arial"/>
+              <a:latin typeface="+mn-lt"/>
             </a:endParaRPr>
           </a:p>
         </txPr>
@@ -524,21 +396,21 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="800" b="0">
+              <a:defRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="404040"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="800" b="0">
+            <a:endParaRPr sz="900" b="0">
               <a:solidFill>
-                <a:srgbClr val="404040"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
-              <a:latin typeface="Arial"/>
+              <a:latin typeface="+mn-lt"/>
             </a:endParaRPr>
           </a:p>
         </txPr>
@@ -552,7 +424,7 @@
   <spPr>
     <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
       <a:solidFill>
-        <a:srgbClr val="BFBFBF"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -569,19 +441,19 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1200" b="1">
+              <a:defRPr sz="1400" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1200" b="1">
+              <a:rPr sz="1400" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:rPr>
               <a:t>Weighted SWOT Scores</a:t>
             </a:r>
@@ -623,21 +495,21 @@
             <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
             <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:pPr>
-                <a:defRPr sz="900" b="1">
+                <a:defRPr sz="900" b="0">
                   <a:solidFill>
-                    <a:srgbClr val="000000"/>
+                    <a:srgbClr val="404040"/>
                   </a:solidFill>
-                  <a:latin typeface="Arial"/>
+                  <a:latin typeface="+mn-lt"/>
                 </a:defRPr>
               </a:pPr>
               <a:r>
                 <a:t/>
               </a:r>
-              <a:endParaRPr sz="900" b="1">
+              <a:endParaRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="404040"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:endParaRPr>
             </a:p>
           </txPr>
@@ -648,7 +520,7 @@
           <showSerName val="0"/>
           <showPercent val="0"/>
         </dLbls>
-        <gapWidth val="60"/>
+        <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -664,7 +536,7 @@
         <spPr>
           <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
             <a:solidFill>
-              <a:srgbClr val="A6A6A6"/>
+              <a:srgbClr val="D9D9D9"/>
             </a:solidFill>
             <a:prstDash val="solid"/>
           </a:ln>
@@ -675,9 +547,9 @@
             <a:pPr>
               <a:defRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
@@ -685,9 +557,9 @@
             </a:r>
             <a:endParaRPr sz="900" b="0">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
-              <a:latin typeface="Arial"/>
+              <a:latin typeface="+mn-lt"/>
             </a:endParaRPr>
           </a:p>
         </txPr>
@@ -726,21 +598,21 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="800" b="0">
+              <a:defRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="404040"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="800" b="0">
+            <a:endParaRPr sz="900" b="0">
               <a:solidFill>
-                <a:srgbClr val="404040"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
-              <a:latin typeface="Arial"/>
+              <a:latin typeface="+mn-lt"/>
             </a:endParaRPr>
           </a:p>
         </txPr>
@@ -754,7 +626,7 @@
   <spPr>
     <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
       <a:solidFill>
-        <a:srgbClr val="BFBFBF"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -771,19 +643,19 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1200" b="1">
+              <a:defRPr sz="1400" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1200" b="1">
+              <a:rPr sz="1400" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:rPr>
               <a:t>Porter's Five Forces: Strength (1 to 5)</a:t>
             </a:r>
@@ -825,21 +697,21 @@
             <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
             <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:pPr>
-                <a:defRPr sz="900" b="1">
+                <a:defRPr sz="900" b="0">
                   <a:solidFill>
-                    <a:srgbClr val="000000"/>
+                    <a:srgbClr val="404040"/>
                   </a:solidFill>
-                  <a:latin typeface="Arial"/>
+                  <a:latin typeface="+mn-lt"/>
                 </a:defRPr>
               </a:pPr>
               <a:r>
                 <a:t/>
               </a:r>
-              <a:endParaRPr sz="900" b="1">
+              <a:endParaRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="404040"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:endParaRPr>
             </a:p>
           </txPr>
@@ -850,7 +722,7 @@
           <showSerName val="0"/>
           <showPercent val="0"/>
         </dLbls>
-        <gapWidth val="60"/>
+        <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -866,7 +738,7 @@
         <spPr>
           <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
             <a:solidFill>
-              <a:srgbClr val="A6A6A6"/>
+              <a:srgbClr val="D9D9D9"/>
             </a:solidFill>
             <a:prstDash val="solid"/>
           </a:ln>
@@ -877,9 +749,9 @@
             <a:pPr>
               <a:defRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
@@ -887,9 +759,9 @@
             </a:r>
             <a:endParaRPr sz="900" b="0">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
-              <a:latin typeface="Arial"/>
+              <a:latin typeface="+mn-lt"/>
             </a:endParaRPr>
           </a:p>
         </txPr>
@@ -928,21 +800,21 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="800" b="0">
+              <a:defRPr sz="900" b="0">
                 <a:solidFill>
-                  <a:srgbClr val="404040"/>
+                  <a:srgbClr val="595959"/>
                 </a:solidFill>
-                <a:latin typeface="Arial"/>
+                <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="800" b="0">
+            <a:endParaRPr sz="900" b="0">
               <a:solidFill>
-                <a:srgbClr val="404040"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
-              <a:latin typeface="Arial"/>
+              <a:latin typeface="+mn-lt"/>
             </a:endParaRPr>
           </a:p>
         </txPr>
@@ -956,7 +828,7 @@
   <spPr>
     <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
       <a:solidFill>
-        <a:srgbClr val="BFBFBF"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -1056,104 +928,46 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1165,173 +979,148 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1342,7 +1131,7 @@
     <col width="96" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PZ NIGERIA LIMITED: COMPANY PROFILE</t>
@@ -1356,7 +1145,6 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1382,12 +1170,12 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Marketing Department, Ilupeju, Lagos</t>
         </is>
@@ -1406,12 +1194,12 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Chief Financial Officer</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Mr Oladare Oresukan</t>
         </is>
@@ -1430,12 +1218,12 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Electrical business</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Air conditioners, fridges and freezers, washing machines</t>
         </is>
@@ -1454,12 +1242,12 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>How it is organised</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Product and brand structure: each brand has its own manager, and shared support teams serve all the brands</t>
         </is>
@@ -1477,78 +1265,77 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>What is in this workbook</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>PESTLE</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Political, Economic, Social, Technological, Legal and Environmental factors, each scored Impact × Likelihood, with a summary and chart per factor</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>SWOT</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Strengths, Weaknesses, Opportunities and Threats in a 2 × 2 matrix</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>SWOT Scoring</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>The SWOT points weighted and rated (IFE and EFE matrices) and the strategy they point to</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Industry Analysis</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Industry overview, Porter's Five Forces and the main competitors</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>The key results from every sheet, and the recommendations</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Blue figures are inputs (ratings and weights) you can change. Black figures are formulas: change any blue figure and every score, summary, chart and conclusion updates.</t>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>The ratings and weights are typed in; everything else is a formula. Change any rating or weight and every score, summary, chart and conclusion updates.</t>
         </is>
       </c>
     </row>
@@ -1560,23 +1347,14 @@
     <mergeCell ref="A15:B15"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 PZ Nigeria Limited - &amp;A - Page &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1587,13 +1365,13 @@
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="54" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PESTLE ANALYSIS: PZ NIGERIA LIMITED</t>
@@ -1607,7 +1385,6 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1624,27 +1401,27 @@
           <t>Effect on PZ Nigeria</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Impact (1-5)</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Likelihood (1-5)</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="H4" s="13" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
@@ -1666,22 +1443,22 @@
           <t>Higher fuel and transport costs; easier access to dollars over time</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="10">
         <f>E5*F5</f>
         <v>20</v>
       </c>
-      <c r="H5" s="14" t="str">
+      <c r="H5" s="9" t="str">
         <f>IF(G5&gt;=16,"High",IF(G5&gt;=9,"Medium","Low"))</f>
         <v>High</v>
       </c>
@@ -1702,22 +1479,22 @@
           <t>Imported raw materials and parts cost more</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="10">
         <f>E6*F6</f>
         <v>12</v>
       </c>
-      <c r="H6" s="14" t="str">
+      <c r="H6" s="9" t="str">
         <f>IF(G6&gt;=16,"High",IF(G6&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
@@ -1738,130 +1515,130 @@
           <t>Uncertainty can delay investment and change the rules</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="10">
         <f>E7*F7</f>
         <v>9</v>
       </c>
-      <c r="H7" s="14" t="str">
+      <c r="H7" s="9" t="str">
         <f>IF(G7&gt;=16,"High",IF(G7&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Economic</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Naira devaluation and FX shortages</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Imported raw materials cost much more; losses on foreign-currency debts</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="19">
+      <c r="G8" s="10">
         <f>E8*F8</f>
         <v>25</v>
       </c>
-      <c r="H8" s="17" t="str">
+      <c r="H8" s="9" t="str">
         <f>IF(G8&gt;=16,"High",IF(G8&gt;=9,"Medium","Low"))</f>
         <v>High</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Economic</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>High inflation</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Shoppers buy less or switch to cheaper brands</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="10">
         <f>E9*F9</f>
         <v>25</v>
       </c>
-      <c r="H9" s="17" t="str">
+      <c r="H9" s="9" t="str">
         <f>IF(G9&gt;=16,"High",IF(G9&gt;=9,"Medium","Low"))</f>
         <v>High</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Economic</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>High interest rates</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Borrowing is expensive; fewer appliances bought on credit</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="10">
         <f>E10*F10</f>
         <v>12</v>
       </c>
-      <c r="H10" s="17" t="str">
+      <c r="H10" s="9" t="str">
         <f>IF(G10&gt;=16,"High",IF(G10&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
@@ -1882,22 +1659,22 @@
           <t>A big and growing market for soaps, detergents and appliances</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Opportunity</t>
         </is>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="10">
         <f>E11*F11</f>
         <v>20</v>
       </c>
-      <c r="H11" s="14" t="str">
+      <c r="H11" s="9" t="str">
         <f>IF(G11&gt;=16,"High",IF(G11&gt;=9,"Medium","Low"))</f>
         <v>High</v>
       </c>
@@ -1918,22 +1695,22 @@
           <t>Demand for smaller, cheaper packs</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Opportunity</t>
         </is>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="10">
         <f>E12*F12</f>
         <v>16</v>
       </c>
-      <c r="H12" s="14" t="str">
+      <c r="H12" s="9" t="str">
         <f>IF(G12&gt;=16,"High",IF(G12&gt;=9,"Medium","Low"))</f>
         <v>High</v>
       </c>
@@ -1954,130 +1731,130 @@
           <t>More demand for soaps and cleaning products</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Opportunity</t>
         </is>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="10">
         <f>E13*F13</f>
         <v>12</v>
       </c>
-      <c r="H13" s="14" t="str">
+      <c r="H13" s="9" t="str">
         <f>IF(G13&gt;=16,"High",IF(G13&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Technological</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Social media and digital marketing</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Cheaper, targeted adverts that reach young buyers</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Opportunity</t>
         </is>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="10">
         <f>E14*F14</f>
         <v>15</v>
       </c>
-      <c r="H14" s="17" t="str">
+      <c r="H14" s="9" t="str">
         <f>IF(G14&gt;=16,"High",IF(G14&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Technological</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>E-commerce and modern retail</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>New ways to sell: online stores and supermarkets</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Opportunity</t>
         </is>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F15" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="19">
+      <c r="G15" s="10">
         <f>E15*F15</f>
         <v>12</v>
       </c>
-      <c r="H15" s="17" t="str">
+      <c r="H15" s="9" t="str">
         <f>IF(G15&gt;=16,"High",IF(G15&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Technological</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Poor power supply</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Factories spend more on diesel and solar; demand for energy-saving appliances</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="19">
+      <c r="G16" s="10">
         <f>E16*F16</f>
         <v>16</v>
       </c>
-      <c r="H16" s="17" t="str">
+      <c r="H16" s="9" t="str">
         <f>IF(G16&gt;=16,"High",IF(G16&gt;=9,"Medium","Low"))</f>
         <v>High</v>
       </c>
@@ -2098,22 +1875,22 @@
           <t>Every product must be registered and meet standards</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="10">
         <f>E17*F17</f>
         <v>15</v>
       </c>
-      <c r="H17" s="14" t="str">
+      <c r="H17" s="9" t="str">
         <f>IF(G17&gt;=16,"High",IF(G17&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
@@ -2134,22 +1911,22 @@
           <t>Adverts need approval; fair prices and clear labels</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="E18" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F18" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G18" s="16">
+      <c r="G18" s="10">
         <f>E18*F18</f>
         <v>8</v>
       </c>
-      <c r="H18" s="14" t="str">
+      <c r="H18" s="9" t="str">
         <f>IF(G18&gt;=16,"High",IF(G18&gt;=9,"Medium","Low"))</f>
         <v>Low</v>
       </c>
@@ -2170,167 +1947,160 @@
           <t>Higher staff costs and new tax rules to follow</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F19" s="15" t="n">
+      <c r="F19" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="16">
+      <c r="G19" s="10">
         <f>E19*F19</f>
         <v>12</v>
       </c>
-      <c r="H19" s="14" t="str">
+      <c r="H19" s="9" t="str">
         <f>IF(G19&gt;=16,"High",IF(G19&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Environmental</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Plastic waste rules</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Must change packaging and pay for recycling (EPR)</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E20" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F20" s="18" t="n">
+      <c r="F20" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="10">
         <f>E20*F20</f>
         <v>12</v>
       </c>
-      <c r="H20" s="17" t="str">
+      <c r="H20" s="9" t="str">
         <f>IF(G20&gt;=16,"High",IF(G20&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Environmental</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Flooding and climate change</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Floods disrupt deliveries and damage stock</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="E21" s="18" t="n">
+      <c r="E21" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F21" s="18" t="n">
+      <c r="F21" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G21" s="19">
+      <c r="G21" s="10">
         <f>E21*F21</f>
         <v>9</v>
       </c>
-      <c r="H21" s="17" t="str">
+      <c r="H21" s="9" t="str">
         <f>IF(G21&gt;=16,"High",IF(G21&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Environmental</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Demand for eco-friendly products</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>A chance to launch greener packs and appliances</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Opportunity</t>
         </is>
       </c>
-      <c r="E22" s="18" t="n">
+      <c r="E22" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="18" t="n">
+      <c r="F22" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="10">
         <f>E22*F22</f>
         <v>6</v>
       </c>
-      <c r="H22" s="17" t="str">
+      <c r="H22" s="9" t="str">
         <f>IF(G22&gt;=16,"High",IF(G22&gt;=9,"Medium","Low"))</f>
         <v>Low</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Average score (all issues)</t>
         </is>
       </c>
-      <c r="B23" s="21" t="n"/>
-      <c r="C23" s="21" t="n"/>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="21" t="n"/>
-      <c r="F23" s="21" t="n"/>
-      <c r="G23" s="22">
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="12">
         <f>AVERAGE(G5:G22)</f>
         <v>14.2222222222222</v>
       </c>
-      <c r="H23" s="23" t="str">
+      <c r="H23" s="10" t="str">
         <f>IF(G23&gt;=16,"High",IF(G23&gt;=9,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>PESTLE summary by factor</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="9" t="n"/>
-      <c r="H25" s="9" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -2338,37 +2108,37 @@
           <t>Factor</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Number of issues (COUNTIF)</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Average score (AVERAGEIF)</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>Highest score</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>High priority</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Threats</t>
         </is>
       </c>
-      <c r="G26" s="13" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>Opportunities</t>
         </is>
       </c>
-      <c r="H26" s="13" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
@@ -2380,66 +2150,66 @@
           <t>Political</t>
         </is>
       </c>
-      <c r="B27" s="14">
+      <c r="B27" s="9">
         <f>COUNTIF($A$5:$A$22,A27)</f>
         <v>3</v>
       </c>
-      <c r="C27" s="24">
+      <c r="C27" s="12">
         <f>AVERAGEIF($A$5:$A$22,A27,$G$5:$G$22)</f>
         <v>13.6666666666667</v>
       </c>
-      <c r="D27" s="14">
+      <c r="D27" s="9">
         <f>SUMPRODUCT(MAX(($A$5:$A$22=A27)*$G$5:$G$22))</f>
         <v>20</v>
       </c>
-      <c r="E27" s="14">
+      <c r="E27" s="9">
         <f>COUNTIFS($A$5:$A$22,A27,$H$5:$H$22,"High")</f>
         <v>1</v>
       </c>
-      <c r="F27" s="14">
+      <c r="F27" s="9">
         <f>COUNTIFS($A$5:$A$22,A27,$D$5:$D$22,"Threat")</f>
         <v>3</v>
       </c>
-      <c r="G27" s="14">
+      <c r="G27" s="9">
         <f>COUNTIFS($A$5:$A$22,A27,$D$5:$D$22,"Opportunity")</f>
         <v>0</v>
       </c>
-      <c r="H27" s="14">
+      <c r="H27" s="9">
         <f>RANK(C27,$C$27:$C$32)</f>
         <v>4</v>
       </c>
     </row>
     <row r="28" ht="21" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Economic</t>
         </is>
       </c>
-      <c r="B28" s="17">
+      <c r="B28" s="9">
         <f>COUNTIF($A$5:$A$22,A28)</f>
         <v>3</v>
       </c>
-      <c r="C28" s="25">
+      <c r="C28" s="12">
         <f>AVERAGEIF($A$5:$A$22,A28,$G$5:$G$22)</f>
         <v>20.6666666666667</v>
       </c>
-      <c r="D28" s="17">
+      <c r="D28" s="9">
         <f>SUMPRODUCT(MAX(($A$5:$A$22=A28)*$G$5:$G$22))</f>
         <v>25</v>
       </c>
-      <c r="E28" s="17">
+      <c r="E28" s="9">
         <f>COUNTIFS($A$5:$A$22,A28,$H$5:$H$22,"High")</f>
         <v>2</v>
       </c>
-      <c r="F28" s="17">
+      <c r="F28" s="9">
         <f>COUNTIFS($A$5:$A$22,A28,$D$5:$D$22,"Threat")</f>
         <v>3</v>
       </c>
-      <c r="G28" s="17">
+      <c r="G28" s="9">
         <f>COUNTIFS($A$5:$A$22,A28,$D$5:$D$22,"Opportunity")</f>
         <v>0</v>
       </c>
-      <c r="H28" s="17">
+      <c r="H28" s="9">
         <f>RANK(C28,$C$27:$C$32)</f>
         <v>1</v>
       </c>
@@ -2450,66 +2220,66 @@
           <t>Social</t>
         </is>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="9">
         <f>COUNTIF($A$5:$A$22,A29)</f>
         <v>3</v>
       </c>
-      <c r="C29" s="24">
+      <c r="C29" s="12">
         <f>AVERAGEIF($A$5:$A$22,A29,$G$5:$G$22)</f>
         <v>16</v>
       </c>
-      <c r="D29" s="14">
+      <c r="D29" s="9">
         <f>SUMPRODUCT(MAX(($A$5:$A$22=A29)*$G$5:$G$22))</f>
         <v>20</v>
       </c>
-      <c r="E29" s="14">
+      <c r="E29" s="9">
         <f>COUNTIFS($A$5:$A$22,A29,$H$5:$H$22,"High")</f>
         <v>2</v>
       </c>
-      <c r="F29" s="14">
+      <c r="F29" s="9">
         <f>COUNTIFS($A$5:$A$22,A29,$D$5:$D$22,"Threat")</f>
         <v>0</v>
       </c>
-      <c r="G29" s="14">
+      <c r="G29" s="9">
         <f>COUNTIFS($A$5:$A$22,A29,$D$5:$D$22,"Opportunity")</f>
         <v>3</v>
       </c>
-      <c r="H29" s="14">
+      <c r="H29" s="9">
         <f>RANK(C29,$C$27:$C$32)</f>
         <v>2</v>
       </c>
     </row>
     <row r="30" ht="21" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Technological</t>
         </is>
       </c>
-      <c r="B30" s="17">
+      <c r="B30" s="9">
         <f>COUNTIF($A$5:$A$22,A30)</f>
         <v>3</v>
       </c>
-      <c r="C30" s="25">
+      <c r="C30" s="12">
         <f>AVERAGEIF($A$5:$A$22,A30,$G$5:$G$22)</f>
         <v>14.3333333333333</v>
       </c>
-      <c r="D30" s="17">
+      <c r="D30" s="9">
         <f>SUMPRODUCT(MAX(($A$5:$A$22=A30)*$G$5:$G$22))</f>
         <v>16</v>
       </c>
-      <c r="E30" s="17">
+      <c r="E30" s="9">
         <f>COUNTIFS($A$5:$A$22,A30,$H$5:$H$22,"High")</f>
         <v>1</v>
       </c>
-      <c r="F30" s="17">
+      <c r="F30" s="9">
         <f>COUNTIFS($A$5:$A$22,A30,$D$5:$D$22,"Threat")</f>
         <v>1</v>
       </c>
-      <c r="G30" s="17">
+      <c r="G30" s="9">
         <f>COUNTIFS($A$5:$A$22,A30,$D$5:$D$22,"Opportunity")</f>
         <v>2</v>
       </c>
-      <c r="H30" s="17">
+      <c r="H30" s="9">
         <f>RANK(C30,$C$27:$C$32)</f>
         <v>3</v>
       </c>
@@ -2520,115 +2290,108 @@
           <t>Legal</t>
         </is>
       </c>
-      <c r="B31" s="14">
+      <c r="B31" s="9">
         <f>COUNTIF($A$5:$A$22,A31)</f>
         <v>3</v>
       </c>
-      <c r="C31" s="24">
+      <c r="C31" s="12">
         <f>AVERAGEIF($A$5:$A$22,A31,$G$5:$G$22)</f>
         <v>11.6666666666667</v>
       </c>
-      <c r="D31" s="14">
+      <c r="D31" s="9">
         <f>SUMPRODUCT(MAX(($A$5:$A$22=A31)*$G$5:$G$22))</f>
         <v>15</v>
       </c>
-      <c r="E31" s="14">
+      <c r="E31" s="9">
         <f>COUNTIFS($A$5:$A$22,A31,$H$5:$H$22,"High")</f>
         <v>0</v>
       </c>
-      <c r="F31" s="14">
+      <c r="F31" s="9">
         <f>COUNTIFS($A$5:$A$22,A31,$D$5:$D$22,"Threat")</f>
         <v>3</v>
       </c>
-      <c r="G31" s="14">
+      <c r="G31" s="9">
         <f>COUNTIFS($A$5:$A$22,A31,$D$5:$D$22,"Opportunity")</f>
         <v>0</v>
       </c>
-      <c r="H31" s="14">
+      <c r="H31" s="9">
         <f>RANK(C31,$C$27:$C$32)</f>
         <v>5</v>
       </c>
     </row>
     <row r="32" ht="21" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Environmental</t>
         </is>
       </c>
-      <c r="B32" s="17">
+      <c r="B32" s="9">
         <f>COUNTIF($A$5:$A$22,A32)</f>
         <v>3</v>
       </c>
-      <c r="C32" s="25">
+      <c r="C32" s="12">
         <f>AVERAGEIF($A$5:$A$22,A32,$G$5:$G$22)</f>
         <v>9</v>
       </c>
-      <c r="D32" s="17">
+      <c r="D32" s="9">
         <f>SUMPRODUCT(MAX(($A$5:$A$22=A32)*$G$5:$G$22))</f>
         <v>12</v>
       </c>
-      <c r="E32" s="17">
+      <c r="E32" s="9">
         <f>COUNTIFS($A$5:$A$22,A32,$H$5:$H$22,"High")</f>
         <v>0</v>
       </c>
-      <c r="F32" s="17">
+      <c r="F32" s="9">
         <f>COUNTIFS($A$5:$A$22,A32,$D$5:$D$22,"Threat")</f>
         <v>2</v>
       </c>
-      <c r="G32" s="17">
+      <c r="G32" s="9">
         <f>COUNTIFS($A$5:$A$22,A32,$D$5:$D$22,"Opportunity")</f>
         <v>1</v>
       </c>
-      <c r="H32" s="17">
+      <c r="H32" s="9">
         <f>RANK(C32,$C$27:$C$32)</f>
         <v>6</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="20" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>All factors</t>
         </is>
       </c>
-      <c r="B33" s="23">
+      <c r="B33" s="10">
         <f>SUM(B27:B32)</f>
         <v>18</v>
       </c>
-      <c r="C33" s="22">
+      <c r="C33" s="12">
         <f>AVERAGE(G5:G22)</f>
         <v>14.2222222222222</v>
       </c>
-      <c r="D33" s="23">
+      <c r="D33" s="10">
         <f>MAX(G5:G22)</f>
         <v>25</v>
       </c>
-      <c r="E33" s="23">
+      <c r="E33" s="10">
         <f>SUM(E27:E32)</f>
         <v>6</v>
       </c>
-      <c r="F33" s="23">
+      <c r="F33" s="10">
         <f>SUM(F27:F32)</f>
         <v>12</v>
       </c>
-      <c r="G33" s="23">
+      <c r="G33" s="10">
         <f>SUM(G27:G32)</f>
         <v>6</v>
       </c>
-      <c r="H33" s="23" t="n"/>
-    </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="H33" s="10" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Key findings</t>
         </is>
       </c>
-      <c r="B35" s="9" t="n"/>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="9" t="n"/>
-      <c r="F35" s="9" t="n"/>
-      <c r="G35" s="9" t="n"/>
-      <c r="H35" s="9" t="n"/>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
@@ -2636,21 +2399,21 @@
           <t>Finding</t>
         </is>
       </c>
-      <c r="B36" s="26" t="n"/>
+      <c r="B36" s="13" t="n"/>
       <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="D36" s="26" t="n"/>
-      <c r="E36" s="26" t="n"/>
-      <c r="F36" s="26" t="n"/>
-      <c r="G36" s="13" t="inlineStr">
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="8" t="inlineStr">
         <is>
           <t>Excel functions</t>
         </is>
       </c>
-      <c r="H36" s="26" t="n"/>
+      <c r="H36" s="13" t="n"/>
     </row>
     <row r="37" ht="21" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -2658,41 +2421,41 @@
           <t>Most important factor</t>
         </is>
       </c>
-      <c r="B37" s="27" t="n"/>
+      <c r="B37" s="11" t="n"/>
       <c r="C37" s="5" t="str">
         <f>INDEX($A$27:$A$32,MATCH(MAX($C$27:$C$32),$C$27:$C$32,0))&amp;" (average score "&amp;TEXT(MAX($C$27:$C$32),"0.0")&amp;")"</f>
         <v>Economic (average score 20.7)</v>
       </c>
-      <c r="D37" s="27" t="n"/>
-      <c r="E37" s="27" t="n"/>
-      <c r="F37" s="27" t="n"/>
-      <c r="G37" s="28" t="inlineStr">
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="9" t="inlineStr">
         <is>
           <t>INDEX, MATCH, MAX</t>
         </is>
       </c>
-      <c r="H37" s="27" t="n"/>
+      <c r="H37" s="11" t="n"/>
     </row>
     <row r="38" ht="21" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Least important factor</t>
         </is>
       </c>
-      <c r="B38" s="29" t="n"/>
-      <c r="C38" s="7" t="str">
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="5" t="str">
         <f>INDEX($A$27:$A$32,MATCH(MIN($C$27:$C$32),$C$27:$C$32,0))&amp;" (average score "&amp;TEXT(MIN($C$27:$C$32),"0.0")&amp;")"</f>
         <v>Environmental (average score 9.0)</v>
       </c>
-      <c r="D38" s="29" t="n"/>
-      <c r="E38" s="29" t="n"/>
-      <c r="F38" s="29" t="n"/>
-      <c r="G38" s="30" t="inlineStr">
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>INDEX, MATCH, MIN</t>
         </is>
       </c>
-      <c r="H38" s="29" t="n"/>
+      <c r="H38" s="11" t="n"/>
     </row>
     <row r="39" ht="21" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -2700,41 +2463,41 @@
           <t>Highest-scoring issue</t>
         </is>
       </c>
-      <c r="B39" s="27" t="n"/>
+      <c r="B39" s="11" t="n"/>
       <c r="C39" s="5" t="str">
         <f>INDEX($B$5:$B$22,MATCH(MAX($G$5:$G$22),$G$5:$G$22,0))&amp;" (score "&amp;MAX($G$5:$G$22)&amp;" of 25)"</f>
         <v>Naira devaluation and FX shortages (score 25 of 25)</v>
       </c>
-      <c r="D39" s="27" t="n"/>
-      <c r="E39" s="27" t="n"/>
-      <c r="F39" s="27" t="n"/>
-      <c r="G39" s="28" t="inlineStr">
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="9" t="inlineStr">
         <is>
           <t>INDEX, MATCH, MAX</t>
         </is>
       </c>
-      <c r="H39" s="27" t="n"/>
+      <c r="H39" s="11" t="n"/>
     </row>
     <row r="40" ht="21" customHeight="1">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>High-priority issues</t>
         </is>
       </c>
-      <c r="B40" s="29" t="n"/>
-      <c r="C40" s="7" t="str">
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="5" t="str">
         <f>COUNTIF($H$5:$H$22,"High")&amp;" of "&amp;COUNTA($A$5:$A$22)&amp;" issues"</f>
         <v>6 of 18 issues</v>
       </c>
-      <c r="D40" s="29" t="n"/>
-      <c r="E40" s="29" t="n"/>
-      <c r="F40" s="29" t="n"/>
-      <c r="G40" s="30" t="inlineStr">
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>COUNTIF, COUNTA</t>
         </is>
       </c>
-      <c r="H40" s="29" t="n"/>
+      <c r="H40" s="11" t="n"/>
     </row>
     <row r="41" ht="21" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -2742,34 +2505,27 @@
           <t>Threats and opportunities</t>
         </is>
       </c>
-      <c r="B41" s="27" t="n"/>
+      <c r="B41" s="11" t="n"/>
       <c r="C41" s="5" t="str">
         <f>COUNTIF($D$5:$D$22,"Threat")&amp;" threats, "&amp;COUNTIF($D$5:$D$22,"Opportunity")&amp;" opportunities"</f>
         <v>12 threats, 6 opportunities</v>
       </c>
-      <c r="D41" s="27" t="n"/>
-      <c r="E41" s="27" t="n"/>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="28" t="inlineStr">
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="9" t="inlineStr">
         <is>
           <t>COUNTIF</t>
         </is>
       </c>
-      <c r="H41" s="27" t="n"/>
-    </row>
-    <row r="43" ht="24" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="H41" s="11" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Chart: average PESTLE score by factor</t>
         </is>
       </c>
-      <c r="B43" s="9" t="n"/>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="9" t="n"/>
-      <c r="E43" s="9" t="n"/>
-      <c r="F43" s="9" t="n"/>
-      <c r="G43" s="9" t="n"/>
-      <c r="H43" s="9" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1"/>
     <row r="45" ht="15" customHeight="1"/>
@@ -2816,16 +2572,8 @@
     <mergeCell ref="A39:B39"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 PZ Nigeria Limited - &amp;A - Page &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -2833,7 +2581,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2845,7 +2592,7 @@
     <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SWOT ANALYSIS: PZ NIGERIA LIMITED</t>
@@ -2859,201 +2606,200 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="31" t="inlineStr"/>
-      <c r="B4" s="32" t="inlineStr">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>HELPFUL</t>
         </is>
       </c>
-      <c r="C4" s="32" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>HARMFUL</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="33" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>INTERNAL</t>
         </is>
       </c>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>STRENGTHS</t>
         </is>
       </c>
-      <c r="C5" s="34" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>WEAKNESSES</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="35" t="n"/>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>1. Well-known brands such as Imperial Leather and Joy</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>1. Waiting for the UK owner's approval can slow work</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="35" t="n"/>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>2. More than 100 years in Nigeria; trusted by buyers</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>2. Too many management levels can cause delays</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="35" t="n"/>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>3. Wide distribution network across Nigeria</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>3. Brands may fight over the same marketing money</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="35" t="n"/>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>4. Each business focuses on its own customers</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>4. Naira problems force hard decisions on imports</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="35" t="n"/>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>5. One manager per brand; shared teams save money</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>5. Prices often higher than local low-cost brands</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="35" t="n"/>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>6. Support from the UK owner (PZ Cussons)</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n"/>
+      <c r="C11" s="5" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="33" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>EXTERNAL</t>
         </is>
       </c>
-      <c r="B12" s="34" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>OPPORTUNITIES</t>
         </is>
       </c>
-      <c r="C12" s="34" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>THREATS</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="35" t="n"/>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>1. Large, young and growing population</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>1. Naira devaluation and foreign-exchange shortages</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="35" t="n"/>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>2. Social media, e-commerce and modern retail</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>2. High inflation reduces what consumers can spend</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="35" t="n"/>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>3. Smaller, affordable packs for shoppers on a budget</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>3. Strong competition and cheap imports</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="35" t="n"/>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>4. Customers left by Unilever and P&amp;G since 2023</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>4. Fake (counterfeit) products</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="35" t="n"/>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>5. Exports to other African countries under AfCFTA</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>5. High energy and transport costs</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="35" t="n"/>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>6. Buying raw materials locally to cut dollar costs</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>6. Policy changes and insecurity</t>
         </is>
@@ -3065,8 +2811,8 @@
           <t>SWOT count</t>
         </is>
       </c>
-      <c r="B20" s="26" t="n"/>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Number of points (COUNTA)</t>
         </is>
@@ -3078,20 +2824,20 @@
           <t>Strengths</t>
         </is>
       </c>
-      <c r="B21" s="27" t="n"/>
-      <c r="C21" s="14">
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="9">
         <f>COUNTA(B6:B11)</f>
         <v>6</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Weaknesses</t>
         </is>
       </c>
-      <c r="B22" s="29" t="n"/>
-      <c r="C22" s="17">
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="9">
         <f>COUNTA(C6:C11)</f>
         <v>5</v>
       </c>
@@ -3102,32 +2848,32 @@
           <t>Opportunities</t>
         </is>
       </c>
-      <c r="B23" s="27" t="n"/>
-      <c r="C23" s="14">
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="9">
         <f>COUNTA(B13:B18)</f>
         <v>6</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Threats</t>
         </is>
       </c>
-      <c r="B24" s="29" t="n"/>
-      <c r="C24" s="17">
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="9">
         <f>COUNTA(C13:C18)</f>
         <v>6</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B25" s="21" t="n"/>
-      <c r="C25" s="23">
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="10">
         <f>SUM(C21:C24)</f>
         <v>23</v>
       </c>
@@ -3146,23 +2892,14 @@
     <mergeCell ref="A5:A11"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 PZ Nigeria Limited - &amp;A - Page &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -3176,7 +2913,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SWOT SCORING: IFE AND EFE MATRICES</t>
@@ -3190,17 +2927,12 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Internal Factor Evaluation (IFE): strengths and weaknesses</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n"/>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -3213,17 +2945,17 @@
           <t>Key factor</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Weighted score</t>
         </is>
@@ -3240,13 +2972,13 @@
           <t>Well-known brands such as Imperial Leather and Joy</t>
         </is>
       </c>
-      <c r="C6" s="36" t="n">
+      <c r="C6" s="16" t="n">
         <v>0.15</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="37">
+      <c r="E6" s="17">
         <f>C6*D6</f>
         <v>0.6</v>
       </c>
@@ -3262,13 +2994,13 @@
           <t>More than 100 years in Nigeria; trusted by buyers</t>
         </is>
       </c>
-      <c r="C7" s="36" t="n">
+      <c r="C7" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="37">
+      <c r="E7" s="17">
         <f>C7*D7</f>
         <v>0.4</v>
       </c>
@@ -3284,13 +3016,13 @@
           <t>Wide distribution network across Nigeria</t>
         </is>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="16" t="n">
         <v>0.12</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="37">
+      <c r="E8" s="17">
         <f>C8*D8</f>
         <v>0.36</v>
       </c>
@@ -3306,13 +3038,13 @@
           <t>Each business focuses on its own customers</t>
         </is>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="C9" s="16" t="n">
         <v>0.08</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="37">
+      <c r="E9" s="17">
         <f>C9*D9</f>
         <v>0.24</v>
       </c>
@@ -3328,13 +3060,13 @@
           <t>One manager per brand; shared teams save money</t>
         </is>
       </c>
-      <c r="C10" s="36" t="n">
+      <c r="C10" s="16" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="17">
         <f>C10*D10</f>
         <v>0.21</v>
       </c>
@@ -3350,182 +3082,178 @@
           <t>Support from the UK owner (PZ Cussons)</t>
         </is>
       </c>
-      <c r="C11" s="36" t="n">
+      <c r="C11" s="16" t="n">
         <v>0.08</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="37">
+      <c r="E11" s="17">
         <f>C11*D11</f>
         <v>0.24</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Weakness</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Waiting for the UK owner's approval can slow work</t>
         </is>
       </c>
-      <c r="C12" s="38" t="n">
+      <c r="C12" s="16" t="n">
         <v>0.08</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="39">
+      <c r="E12" s="17">
         <f>C12*D12</f>
         <v>0.16</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Weakness</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Too many management levels can cause delays</t>
         </is>
       </c>
-      <c r="C13" s="38" t="n">
+      <c r="C13" s="16" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="39">
+      <c r="E13" s="17">
         <f>C13*D13</f>
         <v>0.14</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Weakness</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Brands may fight over the same marketing money</t>
         </is>
       </c>
-      <c r="C14" s="38" t="n">
+      <c r="C14" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="39">
+      <c r="E14" s="17">
         <f>C14*D14</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Weakness</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Naira problems force hard decisions on imports</t>
         </is>
       </c>
-      <c r="C15" s="38" t="n">
+      <c r="C15" s="16" t="n">
         <v>0.12</v>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="39">
+      <c r="E15" s="17">
         <f>C15*D15</f>
         <v>0.12</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Weakness</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Prices often higher than local low-cost brands</t>
         </is>
       </c>
-      <c r="C16" s="38" t="n">
+      <c r="C16" s="16" t="n">
         <v>0.08</v>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="39">
+      <c r="E16" s="17">
         <f>C16*D16</f>
         <v>0.16</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="40">
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="17">
         <f>SUM(C6:C16)</f>
         <v>1</v>
       </c>
-      <c r="D17" s="41" t="n"/>
-      <c r="E17" s="42">
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="17">
         <f>SUM(E6:E16)</f>
         <v>2.73</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Weights check</t>
         </is>
       </c>
-      <c r="B18" s="35" t="n"/>
-      <c r="C18" s="11" t="str">
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="5" t="str">
         <f>IF(ROUND(C17,2)=1,"OK: weights add up to 1.00","Check: weights must add up to 1.00")</f>
         <v>OK: weights add up to 1.00</v>
       </c>
-      <c r="D18" s="35" t="n"/>
-      <c r="E18" s="35" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B19" s="35" t="n"/>
-      <c r="C19" s="10" t="str">
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="4" t="str">
         <f>IF(E17&gt;=2.5,"Above average: strengths outweigh weaknesses","Below average: weaknesses outweigh strengths")</f>
         <v>Above average: strengths outweigh weaknesses</v>
       </c>
-      <c r="D19" s="35" t="n"/>
-      <c r="E19" s="35" t="n"/>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>External Factor Evaluation (EFE): opportunities and threats</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -3538,17 +3266,17 @@
           <t>Key factor</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Weighted score</t>
         </is>
@@ -3565,13 +3293,13 @@
           <t>Large, young and growing population</t>
         </is>
       </c>
-      <c r="C23" s="36" t="n">
+      <c r="C23" s="16" t="n">
         <v>0.12</v>
       </c>
-      <c r="D23" s="15" t="n">
+      <c r="D23" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E23" s="37">
+      <c r="E23" s="17">
         <f>C23*D23</f>
         <v>0.36</v>
       </c>
@@ -3587,13 +3315,13 @@
           <t>Social media, e-commerce and modern retail</t>
         </is>
       </c>
-      <c r="C24" s="36" t="n">
+      <c r="C24" s="16" t="n">
         <v>0.08</v>
       </c>
-      <c r="D24" s="15" t="n">
+      <c r="D24" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="37">
+      <c r="E24" s="17">
         <f>C24*D24</f>
         <v>0.16</v>
       </c>
@@ -3609,13 +3337,13 @@
           <t>Smaller, affordable packs for shoppers on a budget</t>
         </is>
       </c>
-      <c r="C25" s="36" t="n">
+      <c r="C25" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="D25" s="15" t="n">
+      <c r="D25" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E25" s="37">
+      <c r="E25" s="17">
         <f>C25*D25</f>
         <v>0.3</v>
       </c>
@@ -3631,13 +3359,13 @@
           <t>Customers left by Unilever and P&amp;G since 2023</t>
         </is>
       </c>
-      <c r="C26" s="36" t="n">
+      <c r="C26" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="D26" s="15" t="n">
+      <c r="D26" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E26" s="37">
+      <c r="E26" s="17">
         <f>C26*D26</f>
         <v>0.3</v>
       </c>
@@ -3653,13 +3381,13 @@
           <t>Exports to other African countries under AfCFTA</t>
         </is>
       </c>
-      <c r="C27" s="36" t="n">
+      <c r="C27" s="16" t="n">
         <v>0.04</v>
       </c>
-      <c r="D27" s="15" t="n">
+      <c r="D27" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="37">
+      <c r="E27" s="17">
         <f>C27*D27</f>
         <v>0.08</v>
       </c>
@@ -3675,204 +3403,200 @@
           <t>Buying raw materials locally to cut dollar costs</t>
         </is>
       </c>
-      <c r="C28" s="36" t="n">
+      <c r="C28" s="16" t="n">
         <v>0.06</v>
       </c>
-      <c r="D28" s="15" t="n">
+      <c r="D28" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E28" s="37">
+      <c r="E28" s="17">
         <f>C28*D28</f>
         <v>0.12</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Naira devaluation and foreign-exchange shortages</t>
         </is>
       </c>
-      <c r="C29" s="38" t="n">
+      <c r="C29" s="16" t="n">
         <v>0.14</v>
       </c>
-      <c r="D29" s="18" t="n">
+      <c r="D29" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E29" s="39">
+      <c r="E29" s="17">
         <f>C29*D29</f>
         <v>0.28</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>High inflation reduces what consumers can spend</t>
         </is>
       </c>
-      <c r="C30" s="38" t="n">
+      <c r="C30" s="16" t="n">
         <v>0.12</v>
       </c>
-      <c r="D30" s="18" t="n">
+      <c r="D30" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E30" s="39">
+      <c r="E30" s="17">
         <f>C30*D30</f>
         <v>0.24</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Strong competition and cheap imports</t>
         </is>
       </c>
-      <c r="C31" s="38" t="n">
+      <c r="C31" s="16" t="n">
         <v>0.09</v>
       </c>
-      <c r="D31" s="18" t="n">
+      <c r="D31" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E31" s="39">
+      <c r="E31" s="17">
         <f>C31*D31</f>
         <v>0.27</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>Fake (counterfeit) products</t>
         </is>
       </c>
-      <c r="C32" s="38" t="n">
+      <c r="C32" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="D32" s="18" t="n">
+      <c r="D32" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E32" s="39">
+      <c r="E32" s="17">
         <f>C32*D32</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>High energy and transport costs</t>
         </is>
       </c>
-      <c r="C33" s="38" t="n">
+      <c r="C33" s="16" t="n">
         <v>0.06</v>
       </c>
-      <c r="D33" s="18" t="n">
+      <c r="D33" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E33" s="39">
+      <c r="E33" s="17">
         <f>C33*D33</f>
         <v>0.12</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Policy changes and insecurity</t>
         </is>
       </c>
-      <c r="C34" s="38" t="n">
+      <c r="C34" s="16" t="n">
         <v>0.04</v>
       </c>
-      <c r="D34" s="18" t="n">
+      <c r="D34" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E34" s="39">
+      <c r="E34" s="17">
         <f>C34*D34</f>
         <v>0.08</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B35" s="21" t="n"/>
-      <c r="C35" s="40">
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="17">
         <f>SUM(C23:C34)</f>
         <v>1</v>
       </c>
-      <c r="D35" s="41" t="n"/>
-      <c r="E35" s="42">
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="17">
         <f>SUM(E23:E34)</f>
         <v>2.41</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Weights check</t>
         </is>
       </c>
-      <c r="B36" s="35" t="n"/>
-      <c r="C36" s="11" t="str">
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="5" t="str">
         <f>IF(ROUND(C35,2)=1,"OK: weights add up to 1.00","Check: weights must add up to 1.00")</f>
         <v>OK: weights add up to 1.00</v>
       </c>
-      <c r="D36" s="35" t="n"/>
-      <c r="E36" s="35" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B37" s="35" t="n"/>
-      <c r="C37" s="10" t="str">
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="4" t="str">
         <f>IF(E35&gt;=2.5,"Above average: PZ responds well to opportunities and threats","Below average: PZ must respond better to opportunities and threats")</f>
         <v>Below average: PZ must respond better to opportunities and threats</v>
       </c>
-      <c r="D37" s="35" t="n"/>
-      <c r="E37" s="35" t="n"/>
-    </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Strategic position</t>
         </is>
       </c>
-      <c r="B39" s="9" t="n"/>
-      <c r="C39" s="9" t="n"/>
-      <c r="D39" s="9" t="n"/>
-      <c r="E39" s="9" t="n"/>
     </row>
     <row r="40" ht="24" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
@@ -3880,14 +3604,14 @@
           <t>Measure</t>
         </is>
       </c>
-      <c r="B40" s="26" t="n"/>
-      <c r="C40" s="13" t="inlineStr">
+      <c r="B40" s="13" t="n"/>
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="D40" s="26" t="n"/>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="D40" s="13" t="n"/>
+      <c r="E40" s="8" t="inlineStr">
         <is>
           <t>Excel functions</t>
         </is>
@@ -3899,31 +3623,31 @@
           <t>Strengths score</t>
         </is>
       </c>
-      <c r="B41" s="27" t="n"/>
-      <c r="C41" s="37">
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="17">
         <f>SUMIF($A$6:$A$16,"Strength",$E$6:$E$16)</f>
         <v>2.05</v>
       </c>
-      <c r="D41" s="27" t="n"/>
-      <c r="E41" s="28" t="inlineStr">
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="9" t="inlineStr">
         <is>
           <t>SUMIF</t>
         </is>
       </c>
     </row>
     <row r="42" ht="21" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Weaknesses score</t>
         </is>
       </c>
-      <c r="B42" s="29" t="n"/>
-      <c r="C42" s="39">
+      <c r="B42" s="11" t="n"/>
+      <c r="C42" s="17">
         <f>SUMIF($A$6:$A$16,"Weakness",$E$6:$E$16)</f>
         <v>0.68</v>
       </c>
-      <c r="D42" s="29" t="n"/>
-      <c r="E42" s="30" t="inlineStr">
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="9" t="inlineStr">
         <is>
           <t>SUMIF</t>
         </is>
@@ -3935,31 +3659,31 @@
           <t>Opportunities score</t>
         </is>
       </c>
-      <c r="B43" s="27" t="n"/>
-      <c r="C43" s="37">
+      <c r="B43" s="11" t="n"/>
+      <c r="C43" s="17">
         <f>SUMIF($A$23:$A$34,"Opportunity",$E$23:$E$34)</f>
         <v>1.32</v>
       </c>
-      <c r="D43" s="27" t="n"/>
-      <c r="E43" s="28" t="inlineStr">
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="9" t="inlineStr">
         <is>
           <t>SUMIF</t>
         </is>
       </c>
     </row>
     <row r="44" ht="21" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Threats score</t>
         </is>
       </c>
-      <c r="B44" s="29" t="n"/>
-      <c r="C44" s="39">
+      <c r="B44" s="11" t="n"/>
+      <c r="C44" s="17">
         <f>SUMIF($A$23:$A$34,"Threat",$E$23:$E$34)</f>
         <v>1.09</v>
       </c>
-      <c r="D44" s="29" t="n"/>
-      <c r="E44" s="30" t="inlineStr">
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="9" t="inlineStr">
         <is>
           <t>SUMIF</t>
         </is>
@@ -3971,31 +3695,31 @@
           <t>IFE total (internal)</t>
         </is>
       </c>
-      <c r="B45" s="27" t="n"/>
-      <c r="C45" s="37">
+      <c r="B45" s="11" t="n"/>
+      <c r="C45" s="17">
         <f>E17</f>
         <v>2.73</v>
       </c>
-      <c r="D45" s="27" t="n"/>
-      <c r="E45" s="28" t="inlineStr">
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="9" t="inlineStr">
         <is>
           <t>SUM</t>
         </is>
       </c>
     </row>
     <row r="46" ht="21" customHeight="1">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>EFE total (external)</t>
         </is>
       </c>
-      <c r="B46" s="29" t="n"/>
-      <c r="C46" s="39">
+      <c r="B46" s="11" t="n"/>
+      <c r="C46" s="17">
         <f>E35</f>
         <v>2.41</v>
       </c>
-      <c r="D46" s="29" t="n"/>
-      <c r="E46" s="30" t="inlineStr">
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="9" t="inlineStr">
         <is>
           <t>SUM</t>
         </is>
@@ -4007,31 +3731,31 @@
           <t>IE matrix cell</t>
         </is>
       </c>
-      <c r="B47" s="27" t="n"/>
-      <c r="C47" s="16" t="str">
+      <c r="B47" s="11" t="n"/>
+      <c r="C47" s="10" t="str">
         <f>CHOOSE((IF(E35&gt;=3,1,IF(E35&gt;=2,2,3))-1)*3+IF(E17&gt;=3,1,IF(E17&gt;=2,2,3)),"I","II","III","IV","V","VI","VII","VIII","IX")</f>
         <v>V</v>
       </c>
-      <c r="D47" s="27" t="n"/>
-      <c r="E47" s="28" t="inlineStr">
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="9" t="inlineStr">
         <is>
           <t>IF, CHOOSE</t>
         </is>
       </c>
     </row>
     <row r="48" ht="21" customHeight="1">
-      <c r="A48" s="6" t="inlineStr">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="B48" s="29" t="n"/>
-      <c r="C48" s="19" t="str">
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="10" t="str">
         <f>CHOOSE((IF(E35&gt;=3,1,IF(E35&gt;=2,2,3))-1)*3+IF(E17&gt;=3,1,IF(E17&gt;=2,2,3)),"Grow and build","Grow and build","Hold and maintain","Grow and build","Hold and maintain","Harvest or divest","Hold and maintain","Harvest or divest","Harvest or divest")</f>
         <v>Hold and maintain</v>
       </c>
-      <c r="D48" s="29" t="n"/>
-      <c r="E48" s="30" t="inlineStr">
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="9" t="inlineStr">
         <is>
           <t>IF, CHOOSE</t>
         </is>
@@ -4043,28 +3767,24 @@
           <t>Suggested strategies</t>
         </is>
       </c>
-      <c r="B49" s="27" t="n"/>
-      <c r="C49" s="16" t="str">
+      <c r="B49" s="11" t="n"/>
+      <c r="C49" s="10" t="str">
         <f>IF(C48="Hold and maintain","Market penetration and product development",IF(C48="Grow and build","Market penetration, market development and product development","Cut costs or sell weak businesses"))</f>
         <v>Market penetration and product development</v>
       </c>
-      <c r="D49" s="27" t="n"/>
-      <c r="E49" s="28" t="inlineStr">
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t>IF</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="8" t="inlineStr">
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>Chart: weighted SWOT scores</t>
         </is>
       </c>
-      <c r="B51" s="9" t="n"/>
-      <c r="C51" s="9" t="n"/>
-      <c r="D51" s="9" t="n"/>
-      <c r="E51" s="9" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1"/>
     <row r="53" ht="15" customHeight="1"/>
@@ -4122,16 +3842,8 @@
     <mergeCell ref="C49:D49"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 PZ Nigeria Limited - &amp;A - Page &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -4139,7 +3851,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -4152,7 +3863,7 @@
     <col width="62" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>INDUSTRY ANALYSIS: NIGERIAN FMCG AND CONSUMER ELECTRICALS</t>
@@ -4166,16 +3877,12 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Industry overview</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n"/>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -4188,22 +3895,22 @@
           <t>Fast-moving consumer goods (FMCG): personal care (soaps, bathing) and home care (dishwashing), plus consumer electricals</t>
         </is>
       </c>
-      <c r="C5" s="27" t="n"/>
-      <c r="D5" s="27" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Over 200 million people, most of them young: one of Africa's largest consumer markets</t>
         </is>
       </c>
-      <c r="C6" s="29" t="n"/>
-      <c r="D6" s="29" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -4216,22 +3923,22 @@
           <t>Households, reached through distributors, wholesalers, open markets, supermarkets and online stores</t>
         </is>
       </c>
-      <c r="C7" s="27" t="n"/>
-      <c r="D7" s="27" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Key trends</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Prices rising with inflation; shoppers moving to smaller packs and cheaper brands; multinationals cutting local production; more selling online and on social media</t>
         </is>
       </c>
-      <c r="C8" s="29" t="n"/>
-      <c r="D8" s="29" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -4244,18 +3951,15 @@
           <t>Strong brands, low costs, wide distribution, local raw materials and affordable pack sizes</t>
         </is>
       </c>
-      <c r="C9" s="27" t="n"/>
-      <c r="D9" s="27" t="n"/>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Porter's Five Forces</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -4263,12 +3967,12 @@
           <t>Force</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Strength (1-5)</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
@@ -4285,10 +3989,10 @@
           <t>Competitive rivalry</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="16" t="str">
+      <c r="C13" s="10" t="str">
         <f>IF(B13&gt;=4,"High",IF(B13&gt;=3,"Medium","Low"))</f>
         <v>High</v>
       </c>
@@ -4299,19 +4003,19 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Bargaining power of buyers</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="19" t="str">
+      <c r="C14" s="10" t="str">
         <f>IF(B14&gt;=4,"High",IF(B14&gt;=3,"Medium","Low"))</f>
         <v>High</v>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Shoppers are price-sensitive and switch brands easily; big distributors bargain hard</t>
         </is>
@@ -4323,10 +4027,10 @@
           <t>Bargaining power of suppliers</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n">
+      <c r="B15" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="16" t="str">
+      <c r="C15" s="10" t="str">
         <f>IF(B15&gt;=4,"High",IF(B15&gt;=3,"Medium","Low"))</f>
         <v>High</v>
       </c>
@@ -4337,19 +4041,19 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Threat of substitutes</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="19" t="str">
+      <c r="C16" s="10" t="str">
         <f>IF(B16&gt;=4,"High",IF(B16&gt;=3,"Medium","Low"))</f>
         <v>Medium</v>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Cheaper unbranded and local soaps; fans instead of air conditioners</t>
         </is>
@@ -4361,10 +4065,10 @@
           <t>Threat of new entrants</t>
         </is>
       </c>
-      <c r="B17" s="15" t="n">
+      <c r="B17" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="16" t="str">
+      <c r="C17" s="10" t="str">
         <f>IF(B17&gt;=4,"High",IF(B17&gt;=3,"Medium","Low"))</f>
         <v>Low</v>
       </c>
@@ -4375,72 +4079,69 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Average strength</t>
         </is>
       </c>
-      <c r="B18" s="22">
+      <c r="B18" s="12">
         <f>AVERAGE(B13:B17)</f>
         <v>3.6</v>
       </c>
-      <c r="C18" s="23" t="str">
+      <c r="C18" s="10" t="str">
         <f>IF(B18&gt;=3.5,"High",IF(B18&gt;=2.5,"Medium","Low"))</f>
         <v>High</v>
       </c>
-      <c r="D18" s="20" t="str">
+      <c r="D18" s="4" t="str">
         <f>IF(B18&gt;=3.5,"Strong competitive pressure: profits are hard to earn",IF(B18&gt;=2.5,"Moderate competitive pressure","Weak competitive pressure: an attractive industry"))</f>
         <v>Strong competitive pressure: profits are hard to earn</v>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Strongest force</t>
         </is>
       </c>
-      <c r="B19" s="11" t="str">
+      <c r="B19" s="5" t="str">
         <f>INDEX($A$13:$A$17,MATCH(MAX($B$13:$B$17),$B$13:$B$17,0))</f>
         <v>Competitive rivalry</v>
       </c>
-      <c r="C19" s="35" t="n"/>
-      <c r="D19" s="35" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
     </row>
     <row r="20" ht="21" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Weakest force</t>
         </is>
       </c>
-      <c r="B20" s="11" t="str">
+      <c r="B20" s="5" t="str">
         <f>INDEX($A$13:$A$17,MATCH(MIN($B$13:$B$17),$B$13:$B$17,0))</f>
         <v>Threat of new entrants</v>
       </c>
-      <c r="C20" s="35" t="n"/>
-      <c r="D20" s="35" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
     </row>
     <row r="21" ht="21" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Forces rated High</t>
         </is>
       </c>
-      <c r="B21" s="11" t="str">
+      <c r="B21" s="5" t="str">
         <f>COUNTIF($C$13:$C$17,"High")&amp;" of "&amp;COUNTA($A$13:$A$17)</f>
         <v>3 of 5</v>
       </c>
-      <c r="C21" s="35" t="n"/>
-      <c r="D21" s="35" t="n"/>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Main competitors</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -4487,22 +4188,22 @@
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Procter &amp; Gamble</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Ariel, Pampers, Always</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Home care</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Stopped making products in Nigeria; imports only (announced 2023)</t>
         </is>
@@ -4531,22 +4232,22 @@
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Hayat Kimya</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Molfix, Bingo, Familia</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Home care</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Makes products locally; low prices; growing fast</t>
         </is>
@@ -4575,49 +4276,46 @@
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>LG, Samsung, Hisense, Scanfrost</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Air conditioners, fridges, washing machines</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>Strong brands, plus many cheaper imports</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Number of competitors listed</t>
         </is>
       </c>
-      <c r="B31" s="20">
+      <c r="B31" s="4">
         <f>COUNTA(A25:A30)</f>
         <v>6</v>
       </c>
-      <c r="C31" s="21" t="n"/>
-      <c r="D31" s="21" t="n"/>
-    </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Chart: strength of the five forces</t>
         </is>
       </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1"/>
     <row r="35" ht="15" customHeight="1"/>
@@ -4655,16 +4353,8 @@
     <mergeCell ref="B20:D20"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 PZ Nigeria Limited - &amp;A - Page &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -4672,7 +4362,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -4683,7 +4372,7 @@
     <col width="92" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="21" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SUMMARY AND RECOMMENDATIONS</t>
@@ -4697,7 +4386,6 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4722,12 +4410,12 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>PESTLE: highest-scoring issue</t>
         </is>
       </c>
-      <c r="B6" s="7" t="str">
+      <c r="B6" s="5" t="str">
         <f>PESTLE!C39</f>
         <v>Naira devaluation and FX shortages (score 25 of 25)</v>
       </c>
@@ -4744,12 +4432,12 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>SWOT: points listed</t>
         </is>
       </c>
-      <c r="B8" s="7" t="str">
+      <c r="B8" s="5" t="str">
         <f>SWOT!C25&amp;" (strengths "&amp;SWOT!C21&amp;", weaknesses "&amp;SWOT!C22&amp;", opportunities "&amp;SWOT!C23&amp;", threats "&amp;SWOT!C24&amp;")"</f>
         <v>23 (strengths 6, weaknesses 5, opportunities 6, threats 6)</v>
       </c>
@@ -4766,12 +4454,12 @@
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>EFE total (external response)</t>
         </is>
       </c>
-      <c r="B10" s="7" t="str">
+      <c r="B10" s="5" t="str">
         <f>TEXT('SWOT Scoring'!E35,"0.00")&amp;" out of 4. "&amp;'SWOT Scoring'!C37</f>
         <v>2.41 out of 4. Below average: PZ must respond better to opportunities and threats</v>
       </c>
@@ -4788,12 +4476,12 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Five Forces: average strength</t>
         </is>
       </c>
-      <c r="B12" s="7" t="str">
+      <c r="B12" s="5" t="str">
         <f>TEXT('Industry Analysis'!B18,"0.0")&amp;" out of 5. "&amp;'Industry Analysis'!D18</f>
         <v>3.6 out of 5. Strong competitive pressure: profits are hard to earn</v>
       </c>
@@ -4809,13 +4497,12 @@
         <v>Competitive rivalry</v>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Recommendations</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -4842,12 +4529,12 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>2. Sell smaller, affordable packs</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Keeps price-sensitive shoppers buying Imperial Leather, Premier Cool, Joy and Morning Fresh</t>
         </is>
@@ -4866,12 +4553,12 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>4. Win customers competitors left behind</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Use the wide distribution network to fill shelves Unilever and P&amp;G have left</t>
         </is>
@@ -4890,7 +4577,7 @@
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Ratings and weights are the analyst's judgement, based on the company information and public news up to 2025. Check the latest figures (exchange rate, inflation) before presenting.</t>
         </is>
@@ -4904,15 +4591,7 @@
     <mergeCell ref="A15:B15"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 PZ Nigeria Limited - &amp;A - Page &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add the written PZ report and colour the workbook to match
The written analysis (introduction, PESTLE, SWOT with IFE/EFE scoring,
industry analysis with Porter's Five Forces and competitors,
recommendations, conclusion) is a Word document built with docx-js from
the same figures as the deck, in Word 2013 compatibility mode, A4,
Calibri, with the deck's two colours.

The workbook now uses those colours too: dark blue header rows and
titles, orange for the harmful side of the SWOT, High ratings (by
conditional formatting) and the top bar in each chart, and light grey
table lines. validate_strict.py now also checks Word documents.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WToQxHdrdWhM7bKqXvUa59
</commit_message>
<xml_diff>
--- a/pz-analysis/PZ_Nigeria_Analysis.xlsx
+++ b/pz-analysis/PZ_Nigeria_Analysis.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,7 +36,7 @@
       <name val="Calibri"/>
       <family val="2"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color theme="4" tint="-0.499984740745262"/>
       <sz val="14"/>
       <scheme val="minor"/>
     </font>
@@ -52,6 +52,14 @@
       <name val="Calibri"/>
       <family val="2"/>
       <b val="1"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color rgb="00000000"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -60,12 +68,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color theme="4" tint="-0.499984740745262"/>
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -74,8 +82,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-        <bgColor rgb="00D9D9D9"/>
+        <fgColor theme="4" tint="-0.499984740745262"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,23 +101,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color theme="0" tint="-0.249977111117893"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color theme="0" tint="-0.249977111117893"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color theme="0" tint="-0.249977111117893"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color theme="0" tint="-0.249977111117893"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -116,13 +128,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -134,30 +146,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="5" tint="-0.249977111117893"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -269,13 +295,29 @@
           <order val="0"/>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="595959"/>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="50000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
           <cat>
             <numRef>
               <f>'PESTLE'!$A$27:$A$32</f>
@@ -471,13 +513,43 @@
           <order val="0"/>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="595959"/>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="50000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
           <cat>
             <numRef>
               <f>'SWOT Scoring'!$A$41:$A$44</f>
@@ -673,13 +745,29 @@
           <order val="0"/>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="595959"/>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="50000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
           <cat>
             <numRef>
               <f>'Industry Analysis'!$A$13:$A$17</f>
@@ -2571,6 +2659,11 @@
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="A39:B39"/>
   </mergeCells>
+  <conditionalFormatting sqref="H5:H22">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"High"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -2613,14 +2706,14 @@
           <t>HELPFUL</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>HARMFUL</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>INTERNAL</t>
         </is>
@@ -2630,7 +2723,7 @@
           <t>STRENGTHS</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>WEAKNESSES</t>
         </is>
@@ -2711,7 +2804,7 @@
       <c r="C11" s="5" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>EXTERNAL</t>
         </is>
@@ -2721,7 +2814,7 @@
           <t>OPPORTUNITIES</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>THREATS</t>
         </is>
@@ -2972,13 +3065,13 @@
           <t>Well-known brands such as Imperial Leather and Joy</t>
         </is>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="18" t="n">
         <v>0.15</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="19">
         <f>C6*D6</f>
         <v>0.6</v>
       </c>
@@ -2994,13 +3087,13 @@
           <t>More than 100 years in Nigeria; trusted by buyers</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="18" t="n">
         <v>0.1</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="19">
         <f>C7*D7</f>
         <v>0.4</v>
       </c>
@@ -3016,13 +3109,13 @@
           <t>Wide distribution network across Nigeria</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="18" t="n">
         <v>0.12</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="19">
         <f>C8*D8</f>
         <v>0.36</v>
       </c>
@@ -3038,13 +3131,13 @@
           <t>Each business focuses on its own customers</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="18" t="n">
         <v>0.08</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="19">
         <f>C9*D9</f>
         <v>0.24</v>
       </c>
@@ -3060,13 +3153,13 @@
           <t>One manager per brand; shared teams save money</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="18" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="19">
         <f>C10*D10</f>
         <v>0.21</v>
       </c>
@@ -3082,13 +3175,13 @@
           <t>Support from the UK owner (PZ Cussons)</t>
         </is>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="18" t="n">
         <v>0.08</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="19">
         <f>C11*D11</f>
         <v>0.24</v>
       </c>
@@ -3104,13 +3197,13 @@
           <t>Waiting for the UK owner's approval can slow work</t>
         </is>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="18" t="n">
         <v>0.08</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="19">
         <f>C12*D12</f>
         <v>0.16</v>
       </c>
@@ -3126,13 +3219,13 @@
           <t>Too many management levels can cause delays</t>
         </is>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="18" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="17">
+      <c r="E13" s="19">
         <f>C13*D13</f>
         <v>0.14</v>
       </c>
@@ -3148,13 +3241,13 @@
           <t>Brands may fight over the same marketing money</t>
         </is>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="18" t="n">
         <v>0.05</v>
       </c>
       <c r="D14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="17">
+      <c r="E14" s="19">
         <f>C14*D14</f>
         <v>0.1</v>
       </c>
@@ -3170,13 +3263,13 @@
           <t>Naira problems force hard decisions on imports</t>
         </is>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="C15" s="18" t="n">
         <v>0.12</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="19">
         <f>C15*D15</f>
         <v>0.12</v>
       </c>
@@ -3192,13 +3285,13 @@
           <t>Prices often higher than local low-cost brands</t>
         </is>
       </c>
-      <c r="C16" s="16" t="n">
+      <c r="C16" s="18" t="n">
         <v>0.08</v>
       </c>
       <c r="D16" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="19">
         <f>C16*D16</f>
         <v>0.16</v>
       </c>
@@ -3210,12 +3303,12 @@
         </is>
       </c>
       <c r="B17" s="11" t="n"/>
-      <c r="C17" s="17">
+      <c r="C17" s="19">
         <f>SUM(C6:C16)</f>
         <v>1</v>
       </c>
       <c r="D17" s="5" t="n"/>
-      <c r="E17" s="17">
+      <c r="E17" s="19">
         <f>SUM(E6:E16)</f>
         <v>2.73</v>
       </c>
@@ -3293,13 +3386,13 @@
           <t>Large, young and growing population</t>
         </is>
       </c>
-      <c r="C23" s="16" t="n">
+      <c r="C23" s="18" t="n">
         <v>0.12</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="19">
         <f>C23*D23</f>
         <v>0.36</v>
       </c>
@@ -3315,13 +3408,13 @@
           <t>Social media, e-commerce and modern retail</t>
         </is>
       </c>
-      <c r="C24" s="16" t="n">
+      <c r="C24" s="18" t="n">
         <v>0.08</v>
       </c>
       <c r="D24" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="17">
+      <c r="E24" s="19">
         <f>C24*D24</f>
         <v>0.16</v>
       </c>
@@ -3337,13 +3430,13 @@
           <t>Smaller, affordable packs for shoppers on a budget</t>
         </is>
       </c>
-      <c r="C25" s="16" t="n">
+      <c r="C25" s="18" t="n">
         <v>0.1</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E25" s="17">
+      <c r="E25" s="19">
         <f>C25*D25</f>
         <v>0.3</v>
       </c>
@@ -3359,13 +3452,13 @@
           <t>Customers left by Unilever and P&amp;G since 2023</t>
         </is>
       </c>
-      <c r="C26" s="16" t="n">
+      <c r="C26" s="18" t="n">
         <v>0.1</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E26" s="17">
+      <c r="E26" s="19">
         <f>C26*D26</f>
         <v>0.3</v>
       </c>
@@ -3381,13 +3474,13 @@
           <t>Exports to other African countries under AfCFTA</t>
         </is>
       </c>
-      <c r="C27" s="16" t="n">
+      <c r="C27" s="18" t="n">
         <v>0.04</v>
       </c>
       <c r="D27" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="17">
+      <c r="E27" s="19">
         <f>C27*D27</f>
         <v>0.08</v>
       </c>
@@ -3403,13 +3496,13 @@
           <t>Buying raw materials locally to cut dollar costs</t>
         </is>
       </c>
-      <c r="C28" s="16" t="n">
+      <c r="C28" s="18" t="n">
         <v>0.06</v>
       </c>
       <c r="D28" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E28" s="17">
+      <c r="E28" s="19">
         <f>C28*D28</f>
         <v>0.12</v>
       </c>
@@ -3425,13 +3518,13 @@
           <t>Naira devaluation and foreign-exchange shortages</t>
         </is>
       </c>
-      <c r="C29" s="16" t="n">
+      <c r="C29" s="18" t="n">
         <v>0.14</v>
       </c>
       <c r="D29" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E29" s="17">
+      <c r="E29" s="19">
         <f>C29*D29</f>
         <v>0.28</v>
       </c>
@@ -3447,13 +3540,13 @@
           <t>High inflation reduces what consumers can spend</t>
         </is>
       </c>
-      <c r="C30" s="16" t="n">
+      <c r="C30" s="18" t="n">
         <v>0.12</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E30" s="17">
+      <c r="E30" s="19">
         <f>C30*D30</f>
         <v>0.24</v>
       </c>
@@ -3469,13 +3562,13 @@
           <t>Strong competition and cheap imports</t>
         </is>
       </c>
-      <c r="C31" s="16" t="n">
+      <c r="C31" s="18" t="n">
         <v>0.09</v>
       </c>
       <c r="D31" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E31" s="17">
+      <c r="E31" s="19">
         <f>C31*D31</f>
         <v>0.27</v>
       </c>
@@ -3491,13 +3584,13 @@
           <t>Fake (counterfeit) products</t>
         </is>
       </c>
-      <c r="C32" s="16" t="n">
+      <c r="C32" s="18" t="n">
         <v>0.05</v>
       </c>
       <c r="D32" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E32" s="17">
+      <c r="E32" s="19">
         <f>C32*D32</f>
         <v>0.1</v>
       </c>
@@ -3513,13 +3606,13 @@
           <t>High energy and transport costs</t>
         </is>
       </c>
-      <c r="C33" s="16" t="n">
+      <c r="C33" s="18" t="n">
         <v>0.06</v>
       </c>
       <c r="D33" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E33" s="17">
+      <c r="E33" s="19">
         <f>C33*D33</f>
         <v>0.12</v>
       </c>
@@ -3535,13 +3628,13 @@
           <t>Policy changes and insecurity</t>
         </is>
       </c>
-      <c r="C34" s="16" t="n">
+      <c r="C34" s="18" t="n">
         <v>0.04</v>
       </c>
       <c r="D34" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E34" s="17">
+      <c r="E34" s="19">
         <f>C34*D34</f>
         <v>0.08</v>
       </c>
@@ -3553,12 +3646,12 @@
         </is>
       </c>
       <c r="B35" s="11" t="n"/>
-      <c r="C35" s="17">
+      <c r="C35" s="19">
         <f>SUM(C23:C34)</f>
         <v>1</v>
       </c>
       <c r="D35" s="5" t="n"/>
-      <c r="E35" s="17">
+      <c r="E35" s="19">
         <f>SUM(E23:E34)</f>
         <v>2.41</v>
       </c>
@@ -3624,7 +3717,7 @@
         </is>
       </c>
       <c r="B41" s="11" t="n"/>
-      <c r="C41" s="17">
+      <c r="C41" s="19">
         <f>SUMIF($A$6:$A$16,"Strength",$E$6:$E$16)</f>
         <v>2.05</v>
       </c>
@@ -3642,7 +3735,7 @@
         </is>
       </c>
       <c r="B42" s="11" t="n"/>
-      <c r="C42" s="17">
+      <c r="C42" s="19">
         <f>SUMIF($A$6:$A$16,"Weakness",$E$6:$E$16)</f>
         <v>0.68</v>
       </c>
@@ -3660,7 +3753,7 @@
         </is>
       </c>
       <c r="B43" s="11" t="n"/>
-      <c r="C43" s="17">
+      <c r="C43" s="19">
         <f>SUMIF($A$23:$A$34,"Opportunity",$E$23:$E$34)</f>
         <v>1.32</v>
       </c>
@@ -3678,7 +3771,7 @@
         </is>
       </c>
       <c r="B44" s="11" t="n"/>
-      <c r="C44" s="17">
+      <c r="C44" s="19">
         <f>SUMIF($A$23:$A$34,"Threat",$E$23:$E$34)</f>
         <v>1.09</v>
       </c>
@@ -3696,7 +3789,7 @@
         </is>
       </c>
       <c r="B45" s="11" t="n"/>
-      <c r="C45" s="17">
+      <c r="C45" s="19">
         <f>E17</f>
         <v>2.73</v>
       </c>
@@ -3714,7 +3807,7 @@
         </is>
       </c>
       <c r="B46" s="11" t="n"/>
-      <c r="C46" s="17">
+      <c r="C46" s="19">
         <f>E35</f>
         <v>2.41</v>
       </c>
@@ -4352,6 +4445,11 @@
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B20:D20"/>
   </mergeCells>
+  <conditionalFormatting sqref="C13:C17">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"High"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>